<commit_message>
Eliminar registro de prueba ING-000001
</commit_message>
<xml_diff>
--- a/operation_data.xlsx
+++ b/operation_data.xlsx
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1282,76 +1283,6 @@
       <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Comprobante Interno (No Fiscal)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>COMPROBANTE-INTERNO</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>municipalidad de Oncativo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>56-51561651-6</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Facturación Directa</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>PENDIENTE MEDIO DE PAGO</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Factura creada directamente</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4391,43 +4322,6 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-10-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>USR-000001</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ailen Avalle</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ailen Avalle</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$rEh9KiKJbs4LgfYc$936c062e2a6a4806534e0015488307681ba70b4ebf64bf6193ccb690a5a1ecbdee3c830cd844b84339be64925ae643774bdad83bd27733bcb2ea989e27bb735b</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>07/10/2026 16:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: agregada eliminacion de facturas y viajes con reversion contable y ajustes de UI
</commit_message>
<xml_diff>
--- a/operation_data.xlsx
+++ b/operation_data.xlsx
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>2312312312</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1151,33 +1151,18 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>COBRADO</t>
+          <t>PENDIENTE MEDIO DE PAGO</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Transferencia: $2,000,000.00 | Cheque Físico (N° test1, test): $1,000,000.00 | E-Cheq (N° test2, test2): $1,000,000.00 | Cheque Físico (N° test3, test3): $1,000,000.00 - Banco Cordoba</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>REC-000002</t>
-        </is>
+        <v>1000000</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -4680,7 +4665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4797,7 +4782,44 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>USR-000001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ailen Avalle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ailen Avalle</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$wagVsgMFwai9CW1o$16a67cee9ae9a25c26a43d75c2fb07af7a8beb682a21454e6f01c80bbf7abdff7e152de3300a56904332e11dda9ba483fbfc7a68661da9d54a35fa7c3991cd48</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>14/10/2026 21:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: facturacion directa historica, proteccion de tesoreria, soporte solo operario y mejoras visuales
</commit_message>
<xml_diff>
--- a/operation_data.xlsx
+++ b/operation_data.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1015,161 +1015,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Factura A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>00001</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>00001-00000002</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Municipalidad de Carrilobo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>30-99901691-6</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Facturación Directa</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>COBRADO</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Cheque: $1,000,000.00 - Caja Chica Efectivo</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>REC-000001</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Factura creada directamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ING-000002</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Factura A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2312312312</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Municipalidad de Oncativo</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>30-99901691-6</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Facturación Directa</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>PENDIENTE MEDIO DE PAGO</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Factura creada directamente</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1181,7 +1026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1367,91 +1212,6 @@
       <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Factura A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>00001</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>00001-00000002</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Municipalidad de Carrilobo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>30-99901691-6</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Facturación Directa</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>COBRADO</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Cheque: $1,000,000.00 - Caja Chica Efectivo</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>REC-000001</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Factura creada directamente</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1557,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>bancor</t>
+          <t>Bancor</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1820,14 +1580,9 @@
           <t>Disponible</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Cobro de Ingreso ING-000001 - Municipalidad de Carrilobo</t>
+          <t>Cheque en cartera - Municipalidad de Carrilobo</t>
         </is>
       </c>
     </row>
@@ -1885,14 +1640,9 @@
           <t>Disponible</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Cobro de Ingreso ING-000001 - Municipalidad de Carrilobo</t>
+          <t>Cheque en cartera - Municipalidad de Carrilobo</t>
         </is>
       </c>
     </row>
@@ -1950,14 +1700,9 @@
           <t>Disponible</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Cobro de Ingreso ING-000001 - Municipalidad de Carrilobo</t>
+          <t>Cheque en cartera - Municipalidad de Carrilobo</t>
         </is>
       </c>
     </row>
@@ -2015,14 +1760,9 @@
           <t>Disponible</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Cobro de Ingreso ING-000001 - Municipalidad de Carrilobo</t>
+          <t>Cheque en cartera - Municipalidad de Carrilobo</t>
         </is>
       </c>
     </row>
@@ -2080,14 +1820,9 @@
           <t>Disponible</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>ING-000001</t>
-        </is>
-      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Cobro de Ingreso ING-000001 - Municipalidad de Carrilobo</t>
+          <t>Cheque en cartera - Municipalidad de Carrilobo</t>
         </is>
       </c>
     </row>
@@ -2102,7 +1837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2229,6 +1964,60 @@
         <is>
           <t>N° cheque</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ORD-000001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CASA MARGARIA</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Herramientas</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>un destornillador</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Cuenta Corriente 30 días</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4665,7 +4454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4745,7 +4534,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -4782,44 +4571,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>USR-000001</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ailen Avalle</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ailen Avalle</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$wagVsgMFwai9CW1o$16a67cee9ae9a25c26a43d75c2fb07af7a8beb682a21454e6f01c80bbf7abdff7e152de3300a56904332e11dda9ba483fbfc7a68661da9d54a35fa7c3991cd48</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>14/10/2026 21:20</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4984,6 +4736,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CLI-000004</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VS Oncativo SA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>30-70339972-6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Responsable Inscripto</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3572695224</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4995,7 +4784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5126,7 +4915,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5148,7 +4937,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ESCALABILIDAD</t>
+          <t>CARRETON | ESCALABILIDAD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5173,7 +4962,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -5220,7 +5009,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -5267,7 +5056,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -5314,12 +5103,180 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2027-01-05</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>2027-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>UNI-000008</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Camión</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No posee ITV RTO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SRF504</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FORD</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>14.000</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UNI-000009</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Semirremolque</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SQB851</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>KRONE</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2027-02-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UNI-000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Camión</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GIZ913</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FORD</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2027-02-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UNI-000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Semirremolque</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>AF770FI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>VULCANO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2027-04-08</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK8"/>
+  <dimension ref="A1:AK10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6174,6 +6131,257 @@
         <v>0</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EMP-000005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Jonas Gimenez</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>37114897</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>20-37114897-4</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1993-11-11</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Soltero</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>YAPEYU 1231</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>zona 6</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Oncativo</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>3572677448</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AILEN MARIA AVALLE </t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>ESPOSA</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>YAPEYU 1231</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ONCATIVO</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>3572595387</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Chofer de Camión</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Completa</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>E.1</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EMP-000006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AILEN MARIA AVALLE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>40028507</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>27-40028507-7</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1997-02-10</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Soltero</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>YAPEYU 1231</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ZONA 6</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ONCATIVO</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>3572595387</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ailenavalle1@gmail.com</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Banco Nacion</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ailen Maria Avalle </t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>mente.corazon.vida</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Completa</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>E.1</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7510,7 +7718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7611,6 +7819,69 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>Items JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PRE-000001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Municipalidad de Carrilobo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>30-99901691-6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Reparación y Mantenimiento de Maquinaria</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15 días</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Cuenta Corriente</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Presupuesto de servicio</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>[{"id": 1, "tipo": "Servicio", "actividad": "452990 - MANTENIMIENTO Y REPARACI\u00d3N DEL MOTOR N.C.P., MEC\u00c1NICA INTEGRAL", "detalle": "Reparaci\u00f3n y Mantenimiento de Maquinaria", "detalle_trabajo": "Reparaci\u00f3n y Mantenimiento de Maquinaria", "ubicacion": "Municipalidad de Carrilobo", "precio_total": 6000000.0, "total": 6000000.0}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: validacion y sanitizacion de fechas para prevenir años fuera de rango y resiliencia en sincronizacion
</commit_message>
<xml_diff>
--- a/operation_data.xlsx
+++ b/operation_data.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1015,6 +1015,88 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ING-000001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Factura A</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>00001</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>00001-00000001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Municipalidad de Carrilobo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>30-99922610-4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Reparacion de barredora marca BICUPIRO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Pendiente de Cobro</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Factura creada directamente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1026,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1212,6 +1294,88 @@
       <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ING-000001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Factura A</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>00001</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>00001-00000001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Municipalidad de Carrilobo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>30-99922610-4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Reparacion de barredora marca BICUPIRO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Pendiente de Cobro</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Factura creada directamente</t>
         </is>
       </c>
     </row>
@@ -1580,6 +1744,10 @@
           <t>Disponible</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>Cheque en cartera - Municipalidad de Carrilobo</t>
@@ -1640,6 +1808,10 @@
           <t>Disponible</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>Cheque en cartera - Municipalidad de Carrilobo</t>
@@ -1700,6 +1872,10 @@
           <t>Disponible</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Cheque en cartera - Municipalidad de Carrilobo</t>
@@ -1760,6 +1936,10 @@
           <t>Disponible</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>Cheque en cartera - Municipalidad de Carrilobo</t>
@@ -1820,6 +2000,10 @@
           <t>Disponible</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Cheque en cartera - Municipalidad de Carrilobo</t>
@@ -1982,6 +2166,7 @@
           <t>CASA MARGARIA</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Herramientas</t>
@@ -2016,9 +2201,14 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2407,11 +2597,15 @@
           <t>Caja Chica</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2452,11 +2646,15 @@
           <t>Efectivo</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2497,11 +2695,15 @@
           <t>Efectivo</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2542,11 +2744,15 @@
           <t>Transferencia - Banco Cordoba</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2587,11 +2793,15 @@
           <t>Transferencia - Banco Cordoba</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4366,12 +4576,14 @@
           <t>Cheques</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Sincronizado automáticamente con Cartera Cheques</t>
@@ -4534,7 +4746,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4783,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4693,6 +4905,8 @@
           <t>Exento / Estado</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Bulnes 727</t>
@@ -4703,6 +4917,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4730,11 +4945,15 @@
           <t>Exento / Estado</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4767,11 +4986,54 @@
           <t>3572695224</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CLI-000005</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cooperativa de trabajo UsinaEco Ltda</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>33-71631049-9</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Responsable Inscripto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+54 9 2323 58-4820 (Martin)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4908,6 +5170,7 @@
           <t>2023</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -4923,6 +5186,8 @@
           <t>2027-06-25</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4955,6 +5220,7 @@
           <t>2023</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -4970,6 +5236,8 @@
           <t>2027-07-08</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5002,6 +5270,7 @@
           <t>2011</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5017,6 +5286,8 @@
           <t>2027-10-21</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5049,6 +5320,7 @@
           <t>2000</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5064,6 +5336,8 @@
           <t>2027-07-08</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5096,6 +5370,7 @@
           <t>2012</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5111,6 +5386,8 @@
           <t>2027-05-05</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5143,6 +5420,7 @@
           <t>14.000</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5153,6 +5431,9 @@
           <t>2027-01-05</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5165,6 +5446,7 @@
           <t>Semirremolque</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>SQB851</t>
@@ -5180,6 +5462,7 @@
           <t>1994</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5195,6 +5478,8 @@
           <t>2027-02-28</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5207,6 +5492,7 @@
           <t>Camión</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>GIZ913</t>
@@ -5222,6 +5508,7 @@
           <t>2007</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5237,6 +5524,8 @@
           <t>2027-02-28</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5249,6 +5538,7 @@
           <t>Semirremolque</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>AF770FI</t>
@@ -5264,6 +5554,7 @@
           <t>2023</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -5279,6 +5570,8 @@
           <t>2027-04-08</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5550,6 +5843,7 @@
           <t>36479383</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>1992-06-11</t>
@@ -5630,6 +5924,7 @@
           <t>PETAK.2026</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>Chofer de Camión</t>
@@ -5640,11 +5935,14 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr">
         <is>
           <t>E.2, B.2</t>
@@ -5680,6 +5978,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="n">
         <v>0</v>
       </c>
@@ -5703,6 +6002,7 @@
           <t>21404440</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>1970-04-24</t>
@@ -5728,6 +6028,7 @@
           <t>Oncativo</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>omarperotti11@gmail.com</t>
@@ -5773,6 +6074,8 @@
           <t>2850400540094100915328</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>Chofer de Camión</t>
@@ -5783,11 +6086,14 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr">
         <is>
           <t>E.1</t>
@@ -5823,6 +6129,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="n">
         <v>0</v>
       </c>
@@ -5846,6 +6153,7 @@
           <t>32889429</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>1987-06-22</t>
@@ -5871,6 +6179,7 @@
           <t>Oncativo</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Longpab22@gmail.com</t>
@@ -5921,6 +6230,7 @@
           <t>PABLOL.2026</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>Chofer de Camión</t>
@@ -5931,11 +6241,14 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr">
         <is>
           <t>E.1</t>
@@ -5971,6 +6284,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
@@ -5994,6 +6308,7 @@
           <t>24242660</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>1974-10-15</t>
@@ -6089,16 +6404,20 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr">
         <is>
           <t>E.1</t>
         </is>
       </c>
+      <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr">
         <is>
           <t>M</t>
@@ -6124,6 +6443,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="n">
         <v>1100000</v>
       </c>
@@ -6182,6 +6502,7 @@
           <t>3572677448</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t xml:space="preserve">AILEN MARIA AVALLE </t>
@@ -6207,6 +6528,11 @@
           <t>3572595387</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>Chofer de Camión</t>
@@ -6217,16 +6543,20 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr">
         <is>
           <t>E.1</t>
         </is>
       </c>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr">
         <is>
           <t>M</t>
@@ -6252,6 +6582,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="n">
         <v>0</v>
       </c>
@@ -6315,6 +6646,11 @@
           <t>ailenavalle1@gmail.com</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>Banco Nacion</t>
@@ -6325,11 +6661,13 @@
           <t xml:space="preserve">Ailen Maria Avalle </t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>mente.corazon.vida</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
           <t>Administrativo</t>
@@ -6340,16 +6678,20 @@
           <t>Completa</t>
         </is>
       </c>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
           <t>Transferencia Bancaria</t>
         </is>
       </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr">
         <is>
           <t>E.1</t>
         </is>
       </c>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr">
         <is>
           <t>M</t>
@@ -6375,6 +6717,7 @@
           <t>Activo</t>
         </is>
       </c>
+      <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
@@ -6393,7 +6736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6507,9 +6850,24 @@
           <t>Grupo Margaria</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>30-60010614-0</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Combustible</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+54 9 3572 44-6460</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>GRUPOMARGARIA.SA@GMAIL.COM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -6520,11 +6878,14 @@
       <c r="I5" t="n">
         <v>-11050.5</v>
       </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6542,6 +6903,7 @@
           <t>YPF</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Combustible</t>
@@ -6552,6 +6914,7 @@
           <t>3572505350</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6560,11 +6923,14 @@
       <c r="I6" t="n">
         <v>2304571.93</v>
       </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6582,11 +6948,14 @@
           <t>Shell</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Combustible</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6595,6 +6964,7 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -6605,6 +6975,7 @@
           <t>Saldo inicial pendiente de confirmar</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6637,6 +7008,7 @@
           <t>3572617398</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6645,11 +7017,13 @@
       <c r="I8" t="n">
         <v>0</v>
       </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>CESOPOL.CORDOBA</t>
@@ -6700,11 +7074,13 @@
       <c r="I9" t="n">
         <v>0</v>
       </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>0000003100008888777766 / YPF.DIRECTO.ONCATIVO</t>
@@ -6742,6 +7118,7 @@
           <t>+54 9 3584 86-6858 (ANAHI)</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6750,11 +7127,13 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>2850400530094013288211</t>
@@ -6792,6 +7171,7 @@
           <t>+54 9 3572 50-0004</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6800,11 +7180,13 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>TACHA.BOLDO.POLLO</t>
@@ -6855,6 +7237,7 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -6865,6 +7248,7 @@
           <t>Contacto: Alarcon Marina Maricel</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6882,6 +7266,7 @@
           <t>GOMERIA EL ALERO</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Repuestos</t>
@@ -6905,6 +7290,7 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -6915,6 +7301,7 @@
           <t>Contacto: Lorena Fernandez</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6947,6 +7334,7 @@
           <t>+54 9 3572 55-0562</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -6955,11 +7343,13 @@
       <c r="I14" t="n">
         <v>0</v>
       </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>cbaceros</t>
@@ -6997,6 +7387,7 @@
           <t>35715322581</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7005,11 +7396,13 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>0200917301000000455283</t>
@@ -7047,6 +7440,7 @@
           <t>3572607034</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7055,11 +7449,14 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7092,6 +7489,7 @@
           <t>3572612848</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7100,11 +7498,13 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>levissamacro</t>
@@ -7142,6 +7542,7 @@
           <t>3572612848</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7150,11 +7551,13 @@
       <c r="I18" t="n">
         <v>0</v>
       </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>lewissrlmacro</t>
@@ -7192,6 +7595,7 @@
           <t>3535107942</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7200,11 +7604,13 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>AMERICAGIS.BN</t>
@@ -7242,6 +7648,7 @@
           <t>3572593304</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7250,11 +7657,13 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>casagonella</t>
@@ -7292,6 +7701,7 @@
           <t>3572509148</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7300,11 +7710,13 @@
       <c r="I21" t="n">
         <v>0</v>
       </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>VENUS.ANCHO.QUESO</t>
@@ -7327,6 +7739,7 @@
           <t>ADMINISTRACION PUMA</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Combustible</t>
@@ -7337,6 +7750,7 @@
           <t>3572446460</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7345,11 +7759,14 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7377,6 +7794,8 @@
           <t>Servicios</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7385,11 +7804,13 @@
       <c r="I23" t="n">
         <v>0</v>
       </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>CCRAVEROZ</t>
@@ -7427,6 +7848,7 @@
           <t>3572677660</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7435,11 +7857,13 @@
       <c r="I24" t="n">
         <v>0</v>
       </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>JALCER.PINTURERIA</t>
@@ -7472,6 +7896,8 @@
           <t>Repuestos</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7480,11 +7906,13 @@
       <c r="I25" t="n">
         <v>0</v>
       </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>DOCTAREP</t>
@@ -7517,6 +7945,12 @@
           <t>Repuestos</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>+54 9 3515 29-5681 (FRANKO)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Cuenta corriente</t>
@@ -7525,6 +7959,7 @@
       <c r="I26" t="n">
         <v>0</v>
       </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>Activo</t>
@@ -7538,6 +7973,59 @@
       <c r="M26" t="inlineStr">
         <is>
           <t>2850306430094195849291 / MEDIT.DIESEL.SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PROV-000024</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Visca Neumaticos S.R.L</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Visca Naumaticos S.R.L</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>30-70753466-0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>3572 43-6119 (Emiliano)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Cuenta corriente</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>VISCA.ONCATIVO.RIO</t>
         </is>
       </c>
     </row>
@@ -7825,39 +8313,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PRE-000001</t>
+          <t>PRE-000002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Municipalidad de Carrilobo</t>
+          <t>Cooperativa de trabajo UsinaEco Ltda</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30-99901691-6</t>
+          <t>33-71631049-9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Viaje</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Reparación y Mantenimiento de Maquinaria</t>
+          <t>Unidad Chasis Volkswagen 17.220. Traslado desde Luján hasta Oncativo, tiempo de espera en el lugar, y posterior retorno desde Oncativo hasta Luján.</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6000000</v>
+        <v>4500000</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -7874,14 +8362,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Presupuesto de servicio</t>
+          <t>Pago a 30 días</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>[{"id": 1, "tipo": "Servicio", "actividad": "452990 - MANTENIMIENTO Y REPARACI\u00d3N DEL MOTOR N.C.P., MEC\u00c1NICA INTEGRAL", "detalle": "Reparaci\u00f3n y Mantenimiento de Maquinaria", "detalle_trabajo": "Reparaci\u00f3n y Mantenimiento de Maquinaria", "ubicacion": "Municipalidad de Carrilobo", "precio_total": 6000000.0, "total": 6000000.0}]</t>
+          <t>[{"id": 1, "tipo": "Viaje", "actividad": "492290 - SERVICIO DE TRANSPORTE AUTOMOTOR DE CARGAS N.C.P.", "subtipo_granel": "General", "toneladas": "", "km": "1160", "origen": "Luján, Buenos Aires", "destino": "Oncativo, Córdoba", "descripcion": "Unidad Chasis Volkswagen 17.220. Traslado desde Luján hasta Oncativo, tiempo de espera en el lugar, y posterior retorno desde Oncativo hasta Luján.", "detalle_trabajo": "", "ubicacion": "", "horas": "", "neto": 4500000}]</t>
         </is>
       </c>
     </row>

</xml_diff>